<commit_message>
chore(data): sync FEB data 2026-03-30 02:41
</commit_message>
<xml_diff>
--- a/data/3FEB_25_26/clutch_aggregated_25_26_3FEB.xlsx
+++ b/data/3FEB_25_26/clutch_aggregated_25_26_3FEB.xlsx
@@ -4007,67 +4007,67 @@
         </is>
       </c>
       <c r="C48" t="n">
+        <v>11</v>
+      </c>
+      <c r="D48" t="n">
+        <v>31.87</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1912.2</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
         <v>10</v>
-      </c>
-      <c r="D48" t="n">
-        <v>29.17</v>
-      </c>
-      <c r="E48" t="n">
-        <v>1750.2</v>
-      </c>
-      <c r="F48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" t="n">
-        <v>9</v>
       </c>
       <c r="H48" t="n">
         <v>5</v>
       </c>
       <c r="I48" t="n">
+        <v>8</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2</v>
+      </c>
+      <c r="R48" t="n">
+        <v>8</v>
+      </c>
+      <c r="S48" t="n">
+        <v>3</v>
+      </c>
+      <c r="T48" t="n">
+        <v>5</v>
+      </c>
+      <c r="U48" t="n">
+        <v>16.7355820520866</v>
+      </c>
+      <c r="V48" t="n">
         <v>7</v>
       </c>
-      <c r="J48" t="n">
-        <v>3</v>
-      </c>
-      <c r="K48" t="n">
-        <v>1</v>
-      </c>
-      <c r="L48" t="n">
-        <v>1</v>
-      </c>
-      <c r="M48" t="n">
-        <v>0.7222222222222222</v>
-      </c>
-      <c r="N48" t="n">
-        <v>0</v>
-      </c>
-      <c r="O48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>2</v>
-      </c>
-      <c r="R48" t="n">
-        <v>7</v>
-      </c>
-      <c r="S48" t="n">
-        <v>3</v>
-      </c>
-      <c r="T48" t="n">
-        <v>4</v>
-      </c>
-      <c r="U48" t="n">
-        <v>16.33993829276654</v>
-      </c>
-      <c r="V48" t="n">
-        <v>12</v>
-      </c>
       <c r="W48" t="n">
-        <v>11.5597188892698</v>
+        <v>-2.416379039849387</v>
       </c>
     </row>
     <row r="49">
@@ -4082,13 +4082,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>0.05</v>
+        <v>2.25</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -4121,28 +4121,28 @@
         <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q49" t="n">
         <v>0</v>
       </c>
       <c r="R49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U49" t="n">
-        <v>0</v>
+        <v>25.19733333333333</v>
       </c>
       <c r="V49" t="n">
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="W49" t="n">
-        <v>0</v>
+        <v>-145.3466666666667</v>
       </c>
     </row>
     <row r="50">
@@ -4232,13 +4232,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D51" t="n">
-        <v>33.37</v>
+        <v>36.07</v>
       </c>
       <c r="E51" t="n">
-        <v>2002.2</v>
+        <v>2164.2</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -4256,10 +4256,10 @@
         <v>4</v>
       </c>
       <c r="K51" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L51" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M51" t="n">
         <v>0.5</v>
@@ -4271,7 +4271,7 @@
         <v>6</v>
       </c>
       <c r="P51" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q51" t="n">
         <v>2</v>
@@ -4286,13 +4286,13 @@
         <v>2</v>
       </c>
       <c r="U51" t="n">
-        <v>34.30365897512736</v>
+        <v>34.69262822289992</v>
       </c>
       <c r="V51" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="W51" t="n">
-        <v>13.75100389571472</v>
+        <v>1.23825894094816</v>
       </c>
     </row>
     <row r="52">
@@ -4532,13 +4532,13 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D55" t="n">
-        <v>17.58</v>
+        <v>18.73</v>
       </c>
       <c r="E55" t="n">
-        <v>1054.8</v>
+        <v>1123.8</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -4586,13 +4586,13 @@
         <v>3</v>
       </c>
       <c r="U55" t="n">
-        <v>28.70343572241184</v>
+        <v>26.94107848371597</v>
       </c>
       <c r="V55" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="W55" t="n">
-        <v>-2.453202502844144</v>
+        <v>-8.117047517351844</v>
       </c>
     </row>
     <row r="56">
@@ -4607,13 +4607,13 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D56" t="n">
-        <v>4.880000000000001</v>
+        <v>5.380000000000001</v>
       </c>
       <c r="E56" t="n">
-        <v>292.8</v>
+        <v>322.8</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -4667,7 +4667,7 @@
         <v>1</v>
       </c>
       <c r="W56" t="n">
-        <v>49.5580737704918</v>
+        <v>44.95230483271376</v>
       </c>
     </row>
     <row r="57">
@@ -4682,13 +4682,13 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D57" t="n">
-        <v>17.41</v>
+        <v>17.91</v>
       </c>
       <c r="E57" t="n">
-        <v>1044.6</v>
+        <v>1074.6</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -4706,7 +4706,7 @@
         <v>1</v>
       </c>
       <c r="K57" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L57" t="n">
         <v>0</v>
@@ -4736,13 +4736,13 @@
         <v>1</v>
       </c>
       <c r="U57" t="n">
-        <v>10.18131533601379</v>
+        <v>12.68881630374093</v>
       </c>
       <c r="V57" t="n">
         <v>-4</v>
       </c>
       <c r="W57" t="n">
-        <v>-25.38288914417002</v>
+        <v>-24.674265773311</v>
       </c>
     </row>
     <row r="58">
@@ -4757,13 +4757,13 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D58" t="n">
-        <v>33.45</v>
+        <v>35.65</v>
       </c>
       <c r="E58" t="n">
-        <v>2007</v>
+        <v>2139</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
@@ -4811,13 +4811,13 @@
         <v>2</v>
       </c>
       <c r="U58" t="n">
-        <v>24.27728550074739</v>
+        <v>22.7791079943899</v>
       </c>
       <c r="V58" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W58" t="n">
-        <v>3.294364723467865</v>
+        <v>-6.08228611500701</v>
       </c>
     </row>
     <row r="59">
@@ -4832,19 +4832,19 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D59" t="n">
-        <v>4.58</v>
+        <v>6.13</v>
       </c>
       <c r="E59" t="n">
-        <v>274.8</v>
+        <v>367.8</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H59" t="n">
         <v>1</v>
@@ -4862,7 +4862,7 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N59" t="n">
         <v>0</v>
@@ -4886,13 +4886,13 @@
         <v>0</v>
       </c>
       <c r="U59" t="n">
-        <v>27.93668122270742</v>
+        <v>27.38882544861338</v>
       </c>
       <c r="V59" t="n">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="W59" t="n">
-        <v>-99.0589519650655</v>
+        <v>-111.9396411092985</v>
       </c>
     </row>
     <row r="60">
@@ -12032,67 +12032,67 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D155" t="n">
-        <v>27.18</v>
+        <v>29.88</v>
       </c>
       <c r="E155" t="n">
-        <v>1630.8</v>
+        <v>1792.8</v>
       </c>
       <c r="F155" t="n">
         <v>0</v>
       </c>
       <c r="G155" t="n">
+        <v>8</v>
+      </c>
+      <c r="H155" t="n">
+        <v>2</v>
+      </c>
+      <c r="I155" t="n">
+        <v>6</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0</v>
+      </c>
+      <c r="K155" t="n">
+        <v>3</v>
+      </c>
+      <c r="L155" t="n">
+        <v>3</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>2</v>
+      </c>
+      <c r="P155" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>2</v>
+      </c>
+      <c r="R155" t="n">
         <v>7</v>
       </c>
-      <c r="H155" t="n">
-        <v>2</v>
-      </c>
-      <c r="I155" t="n">
-        <v>5</v>
-      </c>
-      <c r="J155" t="n">
-        <v>0</v>
-      </c>
-      <c r="K155" t="n">
-        <v>3</v>
-      </c>
-      <c r="L155" t="n">
-        <v>3</v>
-      </c>
-      <c r="M155" t="n">
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="N155" t="n">
-        <v>0</v>
-      </c>
-      <c r="O155" t="n">
-        <v>2</v>
-      </c>
-      <c r="P155" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q155" t="n">
-        <v>2</v>
-      </c>
-      <c r="R155" t="n">
-        <v>6</v>
-      </c>
       <c r="S155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T155" t="n">
         <v>4</v>
       </c>
       <c r="U155" t="n">
-        <v>21.35193524650479</v>
+        <v>22.04935073627845</v>
       </c>
       <c r="V155" t="n">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="W155" t="n">
-        <v>10.43743929359824</v>
+        <v>23.35664658634538</v>
       </c>
     </row>
     <row r="156">
@@ -12107,28 +12107,28 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D156" t="n">
-        <v>8.52</v>
+        <v>11.22</v>
       </c>
       <c r="E156" t="n">
-        <v>511.2</v>
+        <v>673.2</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
       </c>
       <c r="G156" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H156" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I156" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J156" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K156" t="n">
         <v>2</v>
@@ -12137,7 +12137,7 @@
         <v>1</v>
       </c>
       <c r="M156" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="N156" t="n">
         <v>0</v>
@@ -12152,22 +12152,22 @@
         <v>1</v>
       </c>
       <c r="R156" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S156" t="n">
         <v>1</v>
       </c>
       <c r="T156" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U156" t="n">
-        <v>32.9574882629108</v>
+        <v>39.01745098039216</v>
       </c>
       <c r="V156" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W156" t="n">
-        <v>17.43692488262911</v>
+        <v>50.1577183600713</v>
       </c>
     </row>
     <row r="157">
@@ -12332,13 +12332,13 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D159" t="n">
-        <v>31.49</v>
+        <v>34.19</v>
       </c>
       <c r="E159" t="n">
-        <v>1889.4</v>
+        <v>2051.4</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -12374,25 +12374,25 @@
         <v>2</v>
       </c>
       <c r="Q159" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R159" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="S159" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="T159" t="n">
         <v>4</v>
       </c>
       <c r="U159" t="n">
-        <v>32.96378215306446</v>
+        <v>30.36061713951448</v>
       </c>
       <c r="V159" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="W159" t="n">
-        <v>11.71023181962528</v>
+        <v>22.90032758116408</v>
       </c>
     </row>
     <row r="160">
@@ -12482,67 +12482,67 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D161" t="n">
-        <v>12.18</v>
+        <v>14.88</v>
       </c>
       <c r="E161" t="n">
-        <v>730.8</v>
+        <v>892.8</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
       </c>
       <c r="G161" t="n">
+        <v>10</v>
+      </c>
+      <c r="H161" t="n">
+        <v>3</v>
+      </c>
+      <c r="I161" t="n">
+        <v>4</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" t="n">
+        <v>8</v>
+      </c>
+      <c r="L161" t="n">
+        <v>7</v>
+      </c>
+      <c r="M161" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="n">
+        <v>1</v>
+      </c>
+      <c r="P161" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>3</v>
+      </c>
+      <c r="R161" t="n">
+        <v>2</v>
+      </c>
+      <c r="S161" t="n">
+        <v>1</v>
+      </c>
+      <c r="T161" t="n">
+        <v>1</v>
+      </c>
+      <c r="U161" t="n">
+        <v>55.41617607526882</v>
+      </c>
+      <c r="V161" t="n">
         <v>9</v>
       </c>
-      <c r="H161" t="n">
-        <v>2</v>
-      </c>
-      <c r="I161" t="n">
-        <v>4</v>
-      </c>
-      <c r="J161" t="n">
-        <v>0</v>
-      </c>
-      <c r="K161" t="n">
-        <v>7</v>
-      </c>
-      <c r="L161" t="n">
-        <v>6</v>
-      </c>
-      <c r="M161" t="n">
-        <v>0.2222222222222222</v>
-      </c>
-      <c r="N161" t="n">
-        <v>0</v>
-      </c>
-      <c r="O161" t="n">
-        <v>1</v>
-      </c>
-      <c r="P161" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q161" t="n">
-        <v>3</v>
-      </c>
-      <c r="R161" t="n">
-        <v>2</v>
-      </c>
-      <c r="S161" t="n">
-        <v>1</v>
-      </c>
-      <c r="T161" t="n">
-        <v>1</v>
-      </c>
-      <c r="U161" t="n">
-        <v>58.42123973727422</v>
-      </c>
-      <c r="V161" t="n">
-        <v>4</v>
-      </c>
       <c r="W161" t="n">
-        <v>17.86641215106732</v>
+        <v>42.46101478494624</v>
       </c>
     </row>
     <row r="162">
@@ -12632,19 +12632,19 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D163" t="n">
-        <v>22.73</v>
+        <v>24.01</v>
       </c>
       <c r="E163" t="n">
-        <v>1363.8</v>
+        <v>1440.6</v>
       </c>
       <c r="F163" t="n">
         <v>0</v>
       </c>
       <c r="G163" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H163" t="n">
         <v>4</v>
@@ -12662,7 +12662,7 @@
         <v>3</v>
       </c>
       <c r="M163" t="n">
-        <v>0.4</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="N163" t="n">
         <v>0</v>
@@ -12686,13 +12686,13 @@
         <v>0</v>
       </c>
       <c r="U163" t="n">
-        <v>35.36997800263968</v>
+        <v>33.48436484798001</v>
       </c>
       <c r="V163" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W163" t="n">
-        <v>21.20308402991641</v>
+        <v>20.07272386505623</v>
       </c>
     </row>
     <row r="164">
@@ -12932,19 +12932,19 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D167" t="n">
-        <v>11.8</v>
+        <v>13.22</v>
       </c>
       <c r="E167" t="n">
-        <v>708</v>
+        <v>793.2</v>
       </c>
       <c r="F167" t="n">
         <v>0</v>
       </c>
       <c r="G167" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H167" t="n">
         <v>1</v>
@@ -12962,19 +12962,19 @@
         <v>0</v>
       </c>
       <c r="M167" t="n">
-        <v>0.125</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="N167" t="n">
         <v>0</v>
       </c>
       <c r="O167" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P167" t="n">
         <v>1</v>
       </c>
       <c r="Q167" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R167" t="n">
         <v>3</v>
@@ -12986,13 +12986,13 @@
         <v>1</v>
       </c>
       <c r="U167" t="n">
-        <v>44.45210169491526</v>
+        <v>42.79986384266263</v>
       </c>
       <c r="V167" t="n">
-        <v>-5</v>
+        <v>1</v>
       </c>
       <c r="W167" t="n">
-        <v>-2.724491525423729</v>
+        <v>16.30313161875945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>